<commit_message>
rEvised plot with Jenny and Claude
</commit_message>
<xml_diff>
--- a/data/ontario_leader_approval_polls.xlsx
+++ b/data/ontario_leader_approval_polls.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jennyqu/Library/CloudStorage/OneDrive-WilfridLaurierUniversity/ontarioelection2025v2/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lauriercloud-my.sharepoint.com/personal/skiss_wlu_ca/Documents/projects_folder/Ontario_2025_Github/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{911D96A0-5273-7A40-8226-C43CF1FC337D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{911D96A0-5273-7A40-8226-C43CF1FC337D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C5DE5B7-CE4C-2B47-AEFE-A23F46D38F05}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leader Approval Polls" sheetId="1" r:id="rId1"/>
     <sheet name="Methodology &amp; Search Log" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leader Approval Polls'!$A$1:$I$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leader Approval Polls'!$A$1:$I$79</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="138">
   <si>
     <t>Pollster</t>
   </si>
@@ -198,12 +198,6 @@
     <t>Campaign period; 30% don't know enough</t>
   </si>
   <si>
-    <t>impression</t>
-  </si>
-  <si>
-    <t>Campaign start values reported retrospectively in final campaign poll</t>
-  </si>
-  <si>
     <t>https://abacusdata.ca/ontario-election-2025-campaign-final-poll/</t>
   </si>
   <si>
@@ -315,9 +309,6 @@
     <t>Leger</t>
   </si>
   <si>
-    <t>Highest favourability among leaders tested</t>
-  </si>
-  <si>
     <t>https://leger360.com/in-the-news-ontario-voting-intentions-pcs-lead-may-2026/</t>
   </si>
   <si>
@@ -336,9 +327,6 @@
     <t>2026-06-19</t>
   </si>
   <si>
-    <t>Lowest approval in Liaison's Ontario tracker</t>
-  </si>
-  <si>
     <t>https://press.liaisonstrategies.ca/ontario-liberals-lead-pcs-by-3-as-ford-approval-hits-26/</t>
   </si>
   <si>
@@ -409,6 +397,63 @@
   </si>
   <si>
     <t>For a publication-grade series, fetch each pollster's full PDF tables (Abacus archive, Liaison press releases, Angus Reid detailed tables) rather than relying on release summaries; the CSV flags NA where the summary omitted a figure.</t>
+  </si>
+  <si>
+    <t>Corrected from -9: Abacus chart shows 24% positive, 31% negative, net -7 (article text says -9)</t>
+  </si>
+  <si>
+    <t>Campaign launch poll; chart: 26% positive, 34% negative. Dates, URL and metric corrected Sep 30, 2026</t>
+  </si>
+  <si>
+    <t>https://abacusdata.ca/ontario-election-2025-first-poll-abacus-data/</t>
+  </si>
+  <si>
+    <t>33% favourable, 59% unfavourable (net -26 computed). Highest favourability among leaders tested</t>
+  </si>
+  <si>
+    <t>26% approve, 69% disapprove (net -43 computed). Lowest approval in Liaison's Ontario tracker</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Slide: 34% positive, 43% negative (net computed)</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 35% positive, 45% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 34% positive, 43% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 34% positive, 42% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 34% positive, 45% negative, net -11 (article text says -9)</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Text: 37% positive, 43% negative; trend chart shows -6</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Campaign launch poll; chart: 41% positive, 37% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Campaign launch poll; chart: 28% positive, 28% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 37% positive, 39% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 26% positive, 35% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Text: 44% positive, 33% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 46% positive, 33% negative</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Read from Abacus net-impressions trend chart (Jan 13, 2026 point); not stated in text</t>
+  </si>
+  <si>
+    <t>Added Sep 30, 2026. Chart: 36% positive, 42% negative</t>
   </si>
 </sst>
 </file>
@@ -523,7 +568,7 @@
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -580,6 +625,7 @@
     <xf numFmtId="14" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="2" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -885,7 +931,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -926,7 +972,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -982,291 +1028,291 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="23">
+    <row r="4" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="22">
+        <v>44987</v>
+      </c>
+      <c r="C4" s="22">
+        <v>44989</v>
+      </c>
+      <c r="D4" s="22">
+        <v>44992</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="17">
+        <v>-9</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="23">
         <v>45309</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C5" s="23">
         <v>45314</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D5" s="23">
         <v>45320</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="18">
+      <c r="F5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="18">
         <v>3</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="I5" s="24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="22">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="22">
         <v>45309</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C6" s="22">
         <v>45314</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D6" s="22">
         <v>45320</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="17">
+      <c r="F6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="17">
         <v>4</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="2" t="s">
+      <c r="H6" s="3"/>
+      <c r="I6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="25">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="25">
         <v>45309</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C7" s="25">
         <v>45314</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D7" s="25">
         <v>45320</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="19">
+      <c r="F7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="19">
         <v>-19</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="23">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="23">
         <v>45422</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C8" s="23">
         <v>45427</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D8" s="23">
         <v>45434</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="18">
+      <c r="F8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="18">
         <v>0</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="22">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="22">
         <v>45422</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C9" s="22">
         <v>45427</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D9" s="22">
         <v>45434</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="17">
+      <c r="F9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="17">
         <v>6</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="25">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="25">
         <v>45422</v>
       </c>
-      <c r="C9" s="25">
+      <c r="C10" s="25">
         <v>45427</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D10" s="25">
         <v>45434</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="19">
+      <c r="F10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="19">
         <v>-8</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="6" t="s">
+      <c r="H10" s="8"/>
+      <c r="I10" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="23">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="23">
         <v>45463</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C11" s="23">
         <v>45468</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D11" s="23">
         <v>45473</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="18">
+      <c r="F11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="18">
         <v>-2</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="4" t="s">
+      <c r="H11" s="5"/>
+      <c r="I11" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="22">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="22">
         <v>45463</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C12" s="22">
         <v>45468</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D12" s="22">
         <v>45473</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="17">
+      <c r="F12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="17">
         <v>4</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="23">
-        <v>45489</v>
-      </c>
-      <c r="C12" s="23">
-        <v>45494</v>
-      </c>
-      <c r="D12" s="23">
-        <v>45500</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="18">
-        <v>-6</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="22">
-        <v>45489</v>
-      </c>
-      <c r="C13" s="22">
-        <v>45494</v>
-      </c>
-      <c r="D13" s="22">
-        <v>45500</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="17">
-        <v>-1</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="23">
+        <v>45463</v>
+      </c>
+      <c r="C13" s="23">
+        <v>45468</v>
+      </c>
+      <c r="D13" s="23">
+        <v>45473</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="18">
+        <v>-10</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>32</v>
       </c>
@@ -1289,11 +1335,11 @@
         <v>-37</v>
       </c>
       <c r="H14" s="8"/>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>32</v>
       </c>
@@ -1320,7 +1366,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
@@ -1349,7 +1395,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>14</v>
       </c>
@@ -1378,7 +1424,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -1407,7 +1453,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>14</v>
       </c>
@@ -1436,18 +1482,18 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B20" s="23">
-        <v>45568</v>
+        <v>45489</v>
       </c>
       <c r="C20" s="23">
-        <v>45575</v>
+        <v>45494</v>
       </c>
       <c r="D20" s="23">
-        <v>45580</v>
+        <v>45500</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>19</v>
@@ -1456,25 +1502,27 @@
         <v>11</v>
       </c>
       <c r="G20" s="18">
-        <v>-9</v>
-      </c>
-      <c r="H20" s="5"/>
+        <v>-6</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="I20" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="22">
-        <v>45568</v>
+        <v>45489</v>
       </c>
       <c r="C21" s="22">
-        <v>45575</v>
+        <v>45494</v>
       </c>
       <c r="D21" s="22">
-        <v>45580</v>
+        <v>45500</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>10</v>
@@ -1483,28 +1531,30 @@
         <v>11</v>
       </c>
       <c r="G21" s="17">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3"/>
+        <v>-1</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>31</v>
+      </c>
       <c r="I21" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="23">
-        <v>45596</v>
+        <v>45489</v>
       </c>
       <c r="C22" s="23">
-        <v>45601</v>
+        <v>45494</v>
       </c>
       <c r="D22" s="23">
-        <v>45605</v>
+        <v>45500</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>11</v>
@@ -1512,97 +1562,97 @@
       <c r="G22" s="18">
         <v>-9</v>
       </c>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5" t="s">
+        <v>126</v>
+      </c>
       <c r="I22" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="22">
-        <v>45596</v>
-      </c>
-      <c r="C23" s="22">
-        <v>45601</v>
-      </c>
-      <c r="D23" s="22">
-        <v>45605</v>
-      </c>
-      <c r="E23" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="23">
+        <v>45568</v>
+      </c>
+      <c r="C23" s="23">
+        <v>45575</v>
+      </c>
+      <c r="D23" s="23">
+        <v>45580</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" s="18">
+        <v>-9</v>
+      </c>
+      <c r="H23" s="5"/>
+      <c r="I23" s="24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="22">
+        <v>45568</v>
+      </c>
+      <c r="C24" s="22">
+        <v>45575</v>
+      </c>
+      <c r="D24" s="22">
+        <v>45580</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="17">
-        <v>1</v>
-      </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="23">
-        <v>45624</v>
-      </c>
-      <c r="C24" s="23">
-        <v>45630</v>
-      </c>
-      <c r="D24" s="23">
-        <v>45635</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="18">
-        <v>-7</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="22">
-        <v>45624</v>
-      </c>
-      <c r="C25" s="22">
-        <v>45630</v>
-      </c>
-      <c r="D25" s="22">
-        <v>45635</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="17">
-        <v>3</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="17">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="23">
+        <v>45568</v>
+      </c>
+      <c r="C25" s="23">
+        <v>45575</v>
+      </c>
+      <c r="D25" s="23">
+        <v>45580</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" s="18">
+        <v>-8</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>14</v>
       </c>
@@ -1631,7 +1681,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>14</v>
       </c>
@@ -1660,7 +1710,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>14</v>
       </c>
@@ -1689,47 +1739,47 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B29" s="23">
-        <v>45681</v>
+        <v>45596</v>
       </c>
       <c r="C29" s="23">
-        <v>45682</v>
+        <v>45601</v>
       </c>
       <c r="D29" s="23">
-        <v>45683</v>
+        <v>45605</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="G29" s="18">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B30" s="22">
-        <v>45692</v>
+        <v>45596</v>
       </c>
       <c r="C30" s="22">
-        <v>45694</v>
+        <v>45601</v>
       </c>
       <c r="D30" s="22">
-        <v>45697</v>
+        <v>45605</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>10</v>
@@ -1742,50 +1792,50 @@
       </c>
       <c r="H30" s="3"/>
       <c r="I30" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A31" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B31" s="25">
-        <v>45701</v>
-      </c>
-      <c r="C31" s="25">
-        <v>45703</v>
-      </c>
-      <c r="D31" s="25">
-        <v>45707</v>
-      </c>
-      <c r="E31" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" s="23">
+        <v>45596</v>
+      </c>
+      <c r="C31" s="23">
+        <v>45601</v>
+      </c>
+      <c r="D31" s="23">
+        <v>45605</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="19">
-        <v>-10</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F31" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G31" s="18">
+        <v>-11</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B32" s="23">
-        <v>45701</v>
+        <v>45624</v>
       </c>
       <c r="C32" s="23">
-        <v>45703</v>
+        <v>45630</v>
       </c>
       <c r="D32" s="23">
-        <v>45707</v>
+        <v>45635</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>19</v>
@@ -1794,27 +1844,27 @@
         <v>11</v>
       </c>
       <c r="G32" s="18">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B33" s="22">
-        <v>45701</v>
+        <v>45624</v>
       </c>
       <c r="C33" s="22">
-        <v>45703</v>
+        <v>45630</v>
       </c>
       <c r="D33" s="22">
-        <v>45707</v>
+        <v>45635</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>10</v>
@@ -1823,101 +1873,103 @@
         <v>11</v>
       </c>
       <c r="G33" s="17">
-        <v>4</v>
-      </c>
-      <c r="H33" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="I33" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B34" s="25">
-        <v>45712</v>
-      </c>
-      <c r="C34" s="25">
-        <v>45714</v>
-      </c>
-      <c r="D34" s="25">
-        <v>45714</v>
-      </c>
-      <c r="E34" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="23">
+        <v>45624</v>
+      </c>
+      <c r="C34" s="23">
+        <v>45630</v>
+      </c>
+      <c r="D34" s="23">
+        <v>45635</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G34" s="19">
-        <v>3</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+      <c r="F34" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" s="18">
+        <v>-6</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B35" s="23">
-        <v>45712</v>
+        <v>45679</v>
       </c>
       <c r="C35" s="23">
-        <v>45714</v>
+        <v>45683</v>
       </c>
       <c r="D35" s="23">
-        <v>45714</v>
+        <v>45686</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="G35" s="18">
-        <v>2</v>
+        <v>-8</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>61</v>
+        <v>120</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B36" s="22">
-        <v>45712</v>
-      </c>
-      <c r="C36" s="22">
-        <v>45714</v>
-      </c>
-      <c r="D36" s="22">
-        <v>45714</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G36" s="17">
-        <v>9</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="23">
+        <v>45679</v>
+      </c>
+      <c r="C36" s="23">
+        <v>45683</v>
+      </c>
+      <c r="D36" s="23">
+        <v>45686</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" s="18">
+        <v>4</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
         <v>32</v>
       </c>
@@ -1940,11 +1992,11 @@
         <v>3</v>
       </c>
       <c r="H37" s="8"/>
-      <c r="I37" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I37" s="28" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>32</v>
       </c>
@@ -1967,13 +2019,13 @@
         <v>3</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>32</v>
       </c>
@@ -1997,50 +2049,50 @@
       </c>
       <c r="H39" s="3"/>
       <c r="I39" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B40" s="23">
-        <v>45810</v>
+        <v>45679</v>
       </c>
       <c r="C40" s="23">
-        <v>45813</v>
+        <v>45683</v>
       </c>
       <c r="D40" s="23">
-        <v>45818</v>
+        <v>45686</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G40" s="18">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B41" s="22">
-        <v>45810</v>
+        <v>45692</v>
       </c>
       <c r="C41" s="22">
-        <v>45813</v>
+        <v>45694</v>
       </c>
       <c r="D41" s="22">
-        <v>45818</v>
+        <v>45697</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>10</v>
@@ -2049,85 +2101,83 @@
         <v>11</v>
       </c>
       <c r="G41" s="17">
-        <v>3</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>67</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H41" s="3"/>
       <c r="I41" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B42" s="23">
-        <v>45848</v>
-      </c>
-      <c r="C42" s="23">
-        <v>45853</v>
-      </c>
-      <c r="D42" s="23">
-        <v>45862</v>
-      </c>
-      <c r="E42" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" s="22">
+        <v>45692</v>
+      </c>
+      <c r="C42" s="22">
+        <v>45694</v>
+      </c>
+      <c r="D42" s="22">
+        <v>45697</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" s="17">
+        <v>-2</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" s="22">
+        <v>45692</v>
+      </c>
+      <c r="C43" s="22">
+        <v>45694</v>
+      </c>
+      <c r="D43" s="22">
+        <v>45697</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F42" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G42" s="18">
-        <v>1</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="I42" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B43" s="22">
-        <v>45848</v>
-      </c>
-      <c r="C43" s="22">
-        <v>45853</v>
-      </c>
-      <c r="D43" s="22">
-        <v>45862</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="F43" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G43" s="17">
-        <v>4</v>
+        <v>-9</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>70</v>
+        <v>133</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B44" s="25">
-        <v>45884</v>
+        <v>45701</v>
       </c>
       <c r="C44" s="25">
-        <v>45888</v>
+        <v>45703</v>
       </c>
       <c r="D44" s="25">
-        <v>45900</v>
+        <v>45707</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>22</v>
@@ -2136,25 +2186,27 @@
         <v>11</v>
       </c>
       <c r="G44" s="19">
-        <v>14</v>
-      </c>
-      <c r="H44" s="8"/>
+        <v>-10</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>54</v>
+      </c>
       <c r="I44" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B45" s="23">
-        <v>45884</v>
+        <v>45701</v>
       </c>
       <c r="C45" s="23">
-        <v>45888</v>
+        <v>45703</v>
       </c>
       <c r="D45" s="23">
-        <v>45900</v>
+        <v>45707</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>19</v>
@@ -2163,25 +2215,27 @@
         <v>11</v>
       </c>
       <c r="G45" s="18">
-        <v>-3</v>
-      </c>
-      <c r="H45" s="5"/>
+        <v>-4</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>56</v>
+      </c>
       <c r="I45" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B46" s="22">
-        <v>45884</v>
+        <v>45701</v>
       </c>
       <c r="C46" s="22">
-        <v>45888</v>
+        <v>45703</v>
       </c>
       <c r="D46" s="22">
-        <v>45900</v>
+        <v>45707</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>10</v>
@@ -2190,25 +2244,25 @@
         <v>11</v>
       </c>
       <c r="G46" s="17">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H46" s="3"/>
       <c r="I46" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B47" s="25">
-        <v>45912</v>
+        <v>45712</v>
       </c>
       <c r="C47" s="25">
-        <v>45917</v>
+        <v>45714</v>
       </c>
       <c r="D47" s="25">
-        <v>45923</v>
+        <v>45714</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>22</v>
@@ -2217,27 +2271,27 @@
         <v>11</v>
       </c>
       <c r="G47" s="19">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I47" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+      <c r="I47" s="28" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B48" s="23">
-        <v>45912</v>
+        <v>45712</v>
       </c>
       <c r="C48" s="23">
-        <v>45917</v>
+        <v>45714</v>
       </c>
       <c r="D48" s="23">
-        <v>45923</v>
+        <v>45714</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>19</v>
@@ -2246,27 +2300,27 @@
         <v>11</v>
       </c>
       <c r="G48" s="18">
-        <v>-5</v>
+        <v>2</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+      <c r="I48" s="24" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B49" s="22">
-        <v>45912</v>
+        <v>45712</v>
       </c>
       <c r="C49" s="22">
-        <v>45917</v>
+        <v>45714</v>
       </c>
       <c r="D49" s="22">
-        <v>45923</v>
+        <v>45714</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>10</v>
@@ -2275,137 +2329,143 @@
         <v>11</v>
       </c>
       <c r="G49" s="17">
+        <v>9</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50" s="23">
+        <v>45810</v>
+      </c>
+      <c r="C50" s="23">
+        <v>45813</v>
+      </c>
+      <c r="D50" s="23">
+        <v>45818</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G50" s="18">
+        <v>-2</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51" s="22">
+        <v>45810</v>
+      </c>
+      <c r="C51" s="22">
+        <v>45813</v>
+      </c>
+      <c r="D51" s="22">
+        <v>45818</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G51" s="17">
+        <v>3</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" s="23">
+        <v>45810</v>
+      </c>
+      <c r="C52" s="23">
+        <v>45813</v>
+      </c>
+      <c r="D52" s="23">
+        <v>45818</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" s="18">
+        <v>11</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53" s="23">
+        <v>45848</v>
+      </c>
+      <c r="C53" s="23">
+        <v>45853</v>
+      </c>
+      <c r="D53" s="23">
+        <v>45862</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G53" s="18">
         <v>1</v>
       </c>
-      <c r="H49" s="3"/>
-      <c r="I49" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B50" s="25">
-        <v>45939</v>
-      </c>
-      <c r="C50" s="25">
-        <v>45945</v>
-      </c>
-      <c r="D50" s="25">
-        <v>45951</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="19">
-        <v>8</v>
-      </c>
-      <c r="H50" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="I50" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B51" s="23">
-        <v>45939</v>
-      </c>
-      <c r="C51" s="23">
-        <v>45945</v>
-      </c>
-      <c r="D51" s="23">
-        <v>45951</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F51" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="18">
-        <v>-10</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="I51" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B52" s="22">
-        <v>45939</v>
-      </c>
-      <c r="C52" s="22">
-        <v>45945</v>
-      </c>
-      <c r="D52" s="22">
-        <v>45951</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G52" s="17">
-        <v>-1</v>
-      </c>
-      <c r="H52" s="3"/>
-      <c r="I52" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A53" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B53" s="25">
-        <v>46031</v>
-      </c>
-      <c r="C53" s="25">
-        <v>46035</v>
-      </c>
-      <c r="D53" s="25">
-        <v>46036</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F53" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G53" s="19">
-        <v>4</v>
-      </c>
-      <c r="H53" s="8"/>
-      <c r="I53" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H53" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B54" s="22">
-        <v>46031</v>
+        <v>45848</v>
       </c>
       <c r="C54" s="22">
-        <v>46035</v>
+        <v>45853</v>
       </c>
       <c r="D54" s="22">
-        <v>46036</v>
+        <v>45862</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>10</v>
@@ -2414,14 +2474,16 @@
         <v>11</v>
       </c>
       <c r="G54" s="17">
-        <v>6</v>
-      </c>
-      <c r="H54" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="I54" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
         <v>32</v>
       </c>
@@ -2438,19 +2500,19 @@
         <v>22</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G55" s="16">
         <v>-35</v>
       </c>
       <c r="H55" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
         <v>32</v>
       </c>
@@ -2467,16 +2529,16 @@
         <v>22</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G56" s="16">
         <v>-36</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
@@ -2500,100 +2562,98 @@
       </c>
       <c r="G57" s="15"/>
       <c r="H57" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A58" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B58" s="25">
-        <v>46128</v>
-      </c>
-      <c r="C58" s="25">
-        <v>46133</v>
-      </c>
-      <c r="D58" s="25">
-        <v>46139</v>
-      </c>
-      <c r="E58" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B58" s="23">
+        <v>45848</v>
+      </c>
+      <c r="C58" s="23">
+        <v>45853</v>
+      </c>
+      <c r="D58" s="23">
+        <v>45862</v>
+      </c>
+      <c r="E58" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F58" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G58" s="19">
-        <v>-12</v>
-      </c>
-      <c r="H58" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="I58" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A59" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B59" s="22">
-        <v>46128</v>
-      </c>
-      <c r="C59" s="22">
-        <v>46133</v>
-      </c>
-      <c r="D59" s="22">
-        <v>46139</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G59" s="17">
-        <v>5</v>
-      </c>
-      <c r="H59" s="3"/>
-      <c r="I59" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A60" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B60" s="27">
-        <v>46128</v>
-      </c>
-      <c r="C60" s="27">
-        <v>46133</v>
-      </c>
-      <c r="D60" s="27">
-        <v>46139</v>
-      </c>
-      <c r="E60" s="9" t="s">
+      <c r="F58" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G58" s="18">
+        <v>13</v>
+      </c>
+      <c r="H58" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B59" s="25">
+        <v>45884</v>
+      </c>
+      <c r="C59" s="25">
+        <v>45888</v>
+      </c>
+      <c r="D59" s="25">
+        <v>45900</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G59" s="19">
+        <v>14</v>
+      </c>
+      <c r="H59" s="8"/>
+      <c r="I59" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B60" s="23">
+        <v>45884</v>
+      </c>
+      <c r="C60" s="23">
+        <v>45888</v>
+      </c>
+      <c r="D60" s="23">
+        <v>45900</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G60" s="18">
+        <v>-3</v>
+      </c>
+      <c r="H60" s="5"/>
+      <c r="I60" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="F60" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="G60" s="20">
-        <v>3</v>
-      </c>
-      <c r="H60" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="I60" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="6" t="s">
-        <v>90</v>
       </c>
       <c r="B61" s="25">
         <v>46150</v>
@@ -2610,17 +2670,19 @@
       <c r="F61" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G61" s="16"/>
+      <c r="G61" s="16">
+        <v>-26</v>
+      </c>
       <c r="H61" s="8" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B62" s="22">
         <v>46150</v>
@@ -2640,21 +2702,21 @@
       <c r="G62" s="15"/>
       <c r="H62" s="3"/>
       <c r="I62" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B63" s="22">
-        <v>46185</v>
+        <v>45884</v>
       </c>
       <c r="C63" s="22">
-        <v>46190</v>
+        <v>45888</v>
       </c>
       <c r="D63" s="22">
-        <v>46198</v>
+        <v>45900</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>10</v>
@@ -2663,75 +2725,470 @@
         <v>11</v>
       </c>
       <c r="G63" s="17">
-        <v>6</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>94</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H63" s="3"/>
       <c r="I63" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A64" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B64" s="27">
-        <v>46185</v>
-      </c>
-      <c r="C64" s="27">
-        <v>46190</v>
-      </c>
-      <c r="D64" s="27">
-        <v>46198</v>
-      </c>
-      <c r="E64" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="F64" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="G64" s="20">
-        <v>4</v>
-      </c>
-      <c r="H64" s="10"/>
-      <c r="I64" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B64" s="25">
+        <v>45912</v>
+      </c>
+      <c r="C64" s="25">
+        <v>45917</v>
+      </c>
+      <c r="D64" s="25">
+        <v>45923</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G64" s="19">
+        <v>13</v>
+      </c>
+      <c r="H64" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B65" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C65" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C65" s="6" t="s">
-        <v>96</v>
-      </c>
       <c r="D65" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>22</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="G65" s="7"/>
+        <v>77</v>
+      </c>
+      <c r="G65" s="7">
+        <v>-43</v>
+      </c>
       <c r="H65" s="8" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B66" s="23">
+        <v>45912</v>
+      </c>
+      <c r="C66" s="23">
+        <v>45917</v>
+      </c>
+      <c r="D66" s="23">
+        <v>45923</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" s="18">
+        <v>-5</v>
+      </c>
+      <c r="H66" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B67" s="22">
+        <v>45912</v>
+      </c>
+      <c r="C67" s="22">
+        <v>45917</v>
+      </c>
+      <c r="D67" s="22">
+        <v>45923</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" s="17">
+        <v>1</v>
+      </c>
+      <c r="H67" s="3"/>
+      <c r="I67" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B68" s="25">
+        <v>45939</v>
+      </c>
+      <c r="C68" s="25">
+        <v>45945</v>
+      </c>
+      <c r="D68" s="25">
+        <v>45951</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G68" s="19">
+        <v>8</v>
+      </c>
+      <c r="H68" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B69" s="23">
+        <v>45939</v>
+      </c>
+      <c r="C69" s="23">
+        <v>45945</v>
+      </c>
+      <c r="D69" s="23">
+        <v>45951</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G69" s="18">
+        <v>-10</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I69" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B70" s="22">
+        <v>45939</v>
+      </c>
+      <c r="C70" s="22">
+        <v>45945</v>
+      </c>
+      <c r="D70" s="22">
+        <v>45951</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" s="17">
+        <v>-1</v>
+      </c>
+      <c r="H70" s="3"/>
+      <c r="I70" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B71" s="25">
+        <v>46031</v>
+      </c>
+      <c r="C71" s="25">
+        <v>46035</v>
+      </c>
+      <c r="D71" s="25">
+        <v>46036</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" s="19">
+        <v>4</v>
+      </c>
+      <c r="H71" s="8"/>
+      <c r="I71" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B72" s="22">
+        <v>46031</v>
+      </c>
+      <c r="C72" s="22">
+        <v>46035</v>
+      </c>
+      <c r="D72" s="22">
+        <v>46036</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G72" s="17">
+        <v>6</v>
+      </c>
+      <c r="H72" s="3"/>
+      <c r="I72" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B73" s="25">
+        <v>46031</v>
+      </c>
+      <c r="C73" s="25">
+        <v>46035</v>
+      </c>
+      <c r="D73" s="25">
+        <v>46036</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G73" s="19">
+        <v>-7</v>
+      </c>
+      <c r="H73" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B74" s="25">
+        <v>46128</v>
+      </c>
+      <c r="C74" s="25">
+        <v>46133</v>
+      </c>
+      <c r="D74" s="25">
+        <v>46139</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G74" s="19">
+        <v>-12</v>
+      </c>
+      <c r="H74" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B75" s="22">
+        <v>46128</v>
+      </c>
+      <c r="C75" s="22">
+        <v>46133</v>
+      </c>
+      <c r="D75" s="22">
+        <v>46139</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G75" s="17">
+        <v>5</v>
+      </c>
+      <c r="H75" s="3"/>
+      <c r="I75" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B76" s="27">
+        <v>46128</v>
+      </c>
+      <c r="C76" s="27">
+        <v>46133</v>
+      </c>
+      <c r="D76" s="27">
+        <v>46139</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F76" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G76" s="20">
+        <v>3</v>
+      </c>
+      <c r="H76" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="I76" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B77" s="22">
+        <v>46185</v>
+      </c>
+      <c r="C77" s="22">
+        <v>46190</v>
+      </c>
+      <c r="D77" s="22">
+        <v>46198</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G77" s="17">
+        <v>6</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B78" s="27">
+        <v>46185</v>
+      </c>
+      <c r="C78" s="27">
+        <v>46190</v>
+      </c>
+      <c r="D78" s="27">
+        <v>46198</v>
+      </c>
+      <c r="E78" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F78" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G78" s="20">
+        <v>4</v>
+      </c>
+      <c r="H78" s="10"/>
+      <c r="I78" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B79" s="22">
+        <v>46185</v>
+      </c>
+      <c r="C79" s="22">
+        <v>46190</v>
+      </c>
+      <c r="D79" s="22">
+        <v>46198</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G79" s="17">
+        <v>-6</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I65" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:I79" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Abacus Data"/>
-        <filter val="Angus Reid Institute"/>
+        <filter val="Liaison Strategies"/>
       </filters>
     </filterColumn>
     <filterColumn colId="6">
@@ -2739,10 +3196,18 @@
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I79">
+      <sortCondition ref="B1:B79"/>
+    </sortState>
   </autoFilter>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{7450D684-9714-E84C-9304-E8F860BCF707}"/>
-    <hyperlink ref="I4" r:id="rId2" xr:uid="{3AB980EB-4A43-254A-9708-CE8FB01DC30A}"/>
+    <hyperlink ref="I5" r:id="rId2" xr:uid="{3AB980EB-4A43-254A-9708-CE8FB01DC30A}"/>
+    <hyperlink ref="I23" r:id="rId3" xr:uid="{500EF14E-B784-124C-BE50-B5010FDF1DD6}"/>
+    <hyperlink ref="I47" r:id="rId4" xr:uid="{84D72FF6-B75B-A044-B4D2-C3F47B5DA226}"/>
+    <hyperlink ref="I48" r:id="rId5" xr:uid="{52FC1244-84A8-EA47-8B25-F63766F8281B}"/>
+    <hyperlink ref="I14" r:id="rId6" xr:uid="{0A6CD01C-3E03-B648-A987-6ADB13FDCAA5}"/>
+    <hyperlink ref="I37" r:id="rId7" xr:uid="{84F9A8AB-2A33-6746-8314-A9A187A8FA15}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2758,7 +3223,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
@@ -2766,7 +3231,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -2774,7 +3239,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
@@ -2782,7 +3247,7 @@
     </row>
     <row r="7" spans="1:1" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
@@ -2790,7 +3255,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="13" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
@@ -2798,32 +3263,32 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -2831,7 +3296,7 @@
     </row>
     <row r="18" spans="1:1" ht="42" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
@@ -2839,7 +3304,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
@@ -2847,7 +3312,7 @@
     </row>
     <row r="22" spans="1:1" ht="70" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
@@ -2855,7 +3320,7 @@
     </row>
     <row r="24" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
@@ -2863,7 +3328,7 @@
     </row>
     <row r="26" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
@@ -2871,7 +3336,7 @@
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="13" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
@@ -2879,22 +3344,22 @@
     </row>
     <row r="30" spans="1:1" ht="42" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
@@ -2902,7 +3367,7 @@
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
@@ -2910,7 +3375,7 @@
     </row>
     <row r="37" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
@@ -2922,6 +3387,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ac3b9fd6-5397-4331-80b5-7c5a2866cf32" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca995a21-83b3-4c88-8adc-eb51702602b6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100112BD49B8415EA40AAA82944A2852CF3" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="85bfba03f2d7fb09f12fe1445cdb1c8a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ca995a21-83b3-4c88-8adc-eb51702602b6" xmlns:ns3="24078387-fe64-4381-a17d-4cff50d95c75" xmlns:ns4="ac3b9fd6-5397-4331-80b5-7c5a2866cf32" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e25cba0a053820b8ca3d1dafae5f02b9" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="ca995a21-83b3-4c88-8adc-eb51702602b6"/>
@@ -3187,17 +3663,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ac3b9fd6-5397-4331-80b5-7c5a2866cf32" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca995a21-83b3-4c88-8adc-eb51702602b6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3208,6 +3673,24 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03BBA9D4-EA81-4FA4-B015-26F6FB600C4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="ac3b9fd6-5397-4331-80b5-7c5a2866cf32"/>
+    <ds:schemaRef ds:uri="ca995a21-83b3-4c88-8adc-eb51702602b6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="24078387-fe64-4381-a17d-4cff50d95c75"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE5F2CD3-0D9B-46DA-AA32-C3E396BA599C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3227,21 +3710,16 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03BBA9D4-EA81-4FA4-B015-26F6FB600C4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ac3b9fd6-5397-4331-80b5-7c5a2866cf32"/>
-    <ds:schemaRef ds:uri="ca995a21-83b3-4c88-8adc-eb51702602b6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{873A1BFF-A56D-42B8-BCEE-7B764FE083FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{b45a5125-b298-46bc-8b89-ea5a7343fde8}" enabled="0" method="" siteId="{b45a5125-b298-46bc-8b89-ea5a7343fde8}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>